<commit_message>
Refine school calendar display and merged ranges
</commit_message>
<xml_diff>
--- a/kalendarz_dzienny_role_2026_2027.xlsx
+++ b/kalendarz_dzienny_role_2026_2027.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/maciejnajwer/Library/CloudStorage/OneDrive-ZESPÓŁSZKÓŁZAWODOWYCHNR5/zastepstwa-main/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BC837BE9-1702-8947-818F-DDAA4F7DB7B7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{842D50E0-D205-974B-AE4C-3EA432C6215B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="600" windowWidth="34200" windowHeight="19540" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2100" yWindow="600" windowWidth="34200" windowHeight="19540" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Kalendarz dzienny" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="522" uniqueCount="162">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="519" uniqueCount="159">
   <si>
     <t>data</t>
   </si>
@@ -163,9 +163,6 @@
     <t>KLASY 5 TECHNIKUM: wychowawcy klas - złożenie zestawień klasyfikacyjnych / 3 SEMESTR BS II st.: złożenie zestawienia klasyfikacyjnego</t>
   </si>
   <si>
-    <t>15:00 - RADA PEDAGOGICZNA: 1) klasyfikacyjna: KLASY 5 TECHNIKUM oraz 3 SEMESTR BS II st. / 2) szkoleniowa: szkolenie z procedur egzaminu zawodowego</t>
-  </si>
-  <si>
     <t>KLASY 5 TECHNIKUM: zakończenie I półrocza; / 3 SEMESTR BS II st.: zakończenie semestru</t>
   </si>
   <si>
@@ -182,21 +179,12 @@
   </si>
   <si>
     <t>1 SEMESTR BS II st.: złożenie zestawienia klasyfikacyjnego</t>
-  </si>
-  <si>
-    <t>15:00 - RADA PEDAGOGICZNA: 1) klasyfikacyjna: KLASY 1-4 TECHNIKUM, KLASY 1-3 BS I st., 1 SEMESTR BS II st.</t>
   </si>
   <si>
     <t>KLASY 1-4 TECHNIKUM, KLASY 1-3 BS I st.: zakończenie I półrocza / 1 SEMESTR BS II st.: zakończenie semestru
 16:30 - KLASY 1-4 TECHNIKUM, KLASY 1-3 BS I st.: wychowawcy klas - zebrania z rodzicami na zakończenie I półrocza</t>
   </si>
   <si>
-    <t>15:00 - RADA PEDAGOGICZNA: 1) plenarna: podsumowanie I półrocza</t>
-  </si>
-  <si>
-    <t>15:00 - RADA PEDAGOGICZNA: 1) szkoleniowa</t>
-  </si>
-  <si>
     <t>4 SEMESTR BS II st.: poinformowanie słuchaczy (w tym rodziców niepełnoletnich słuchaczy) poprzez wpis do dziennika KOLUMNA "egzamin semestralny" - tak/nie, czy spełniają warunki dopuszczenia do egzaminu semestralnego (co najmniej 50% obecności oraz pozytywne oceny bieżące)</t>
   </si>
   <si>
@@ -212,9 +200,6 @@
     <t>4 SEMESTR BS II st.: złożenie zestawienia klasyfikacyjnego</t>
   </si>
   <si>
-    <t>15:00 - RADA PEDAGOGICZNA: 1) klasyfikacyjna: KLASY 5 TECHNIKUM oraz 4 SEMESTR BS II st. / 2) szkoleniowa: szkolenie z procedur egzaminu maturalnego</t>
-  </si>
-  <si>
     <t>KLASY 5 TECHNIKUM oraz 4 SEMESTR BS II st.: zakończenie roku szkolnego</t>
   </si>
   <si>
@@ -230,9 +215,6 @@
     <t>2 SEMESTR BS II st.: poinformowanie słuchaczy (w tym rodziców niepełnoletnich słuchaczy) poprzez wpis do dziennika KOLUMNA "egzamin semestralny" - tak/nie, czy spełniają warunki dopuszczenia do egzaminu semestralnego (co najmniej 50% obecności oraz pozytywne oceny bieżące)</t>
   </si>
   <si>
-    <t>15:00 - RADA PEDAGOGICZNA: 1) szkoleniowa: szkolenie z procedur egzaminów zawodowych</t>
-  </si>
-  <si>
     <t>KLASY 1-4 TECHNIKUM, KLASY 1-3 BS I st.: wystawienie proponowanych ocen rocznych</t>
   </si>
   <si>
@@ -252,9 +234,6 @@
   </si>
   <si>
     <t>RADA PEDAGOGICZNA: godz. do ustalenia / 1) klasyfikacyjna: KLASY 1-4 TECHNIKUM, KLASY 1-3 BS I st., 2 SEMESTR BS II st.</t>
-  </si>
-  <si>
-    <t>09:00 - RADA PEDAGOGICZNA: 31 sierpnia 2027 r. / 1) klasyfikacyjna: klasyfikacja uczniów po egzaminach poprawkowych / 2) plenarna: podsumowanie roku szkolnego 2026/2027 / 3) inauguracyjna: rozpoczynająca rok szkolny 2027/2028</t>
   </si>
   <si>
     <t>15:00/16:00 - RADA PEDAGOGICZNA: przedstawienie planu nadzoru pedagogicznego na rok szkolny 2026/2027</t>
@@ -374,119 +353,6 @@
 Powód: praktyka zawodowa u pracodawcy – klasy 3 Technikum nie mają zajęć w szkole; pozostałe klasy uczą się normalnie.</t>
   </si>
   <si>
-    <t>Zimowa przerwa świąteczna – 23.12.2026–3.01.2027 (dzień 1 z 12)
-Powód: przerwa świąteczna przewidziana w organizacji roku szkolnego – brak zajęć dydaktyczno-wychowawczych dla wszystkich klas.</t>
-  </si>
-  <si>
-    <t>Zimowa przerwa świąteczna – 23.12.2026–3.01.2027 (dzień 2 z 12)
-Powód: przerwa świąteczna przewidziana w organizacji roku szkolnego – brak zajęć dydaktyczno-wychowawczych dla wszystkich klas.</t>
-  </si>
-  <si>
-    <t>Zimowa przerwa świąteczna – 23.12.2026–3.01.2027 (dzień 3 z 12)
-Powód: przerwa świąteczna przewidziana w organizacji roku szkolnego – brak zajęć dydaktyczno-wychowawczych dla wszystkich klas.</t>
-  </si>
-  <si>
-    <t>Zimowa przerwa świąteczna – 23.12.2026–3.01.2027 (dzień 4 z 12) · weekend
-Powód: przerwa świąteczna przewidziana w organizacji roku szkolnego – brak zajęć dydaktyczno-wychowawczych dla wszystkich klas.</t>
-  </si>
-  <si>
-    <t>Zimowa przerwa świąteczna – 23.12.2026–3.01.2027 (dzień 5 z 12) · weekend
-Powód: przerwa świąteczna przewidziana w organizacji roku szkolnego – brak zajęć dydaktyczno-wychowawczych dla wszystkich klas.</t>
-  </si>
-  <si>
-    <t>Zimowa przerwa świąteczna – 23.12.2026–3.01.2027 (dzień 6 z 12)
-Powód: przerwa świąteczna przewidziana w organizacji roku szkolnego – brak zajęć dydaktyczno-wychowawczych dla wszystkich klas.</t>
-  </si>
-  <si>
-    <t>Zimowa przerwa świąteczna – 23.12.2026–3.01.2027 (dzień 7 z 12)
-Powód: przerwa świąteczna przewidziana w organizacji roku szkolnego – brak zajęć dydaktyczno-wychowawczych dla wszystkich klas.</t>
-  </si>
-  <si>
-    <t>Zimowa przerwa świąteczna – 23.12.2026–3.01.2027 (dzień 8 z 12)
-Powód: przerwa świąteczna przewidziana w organizacji roku szkolnego – brak zajęć dydaktyczno-wychowawczych dla wszystkich klas.</t>
-  </si>
-  <si>
-    <t>Zimowa przerwa świąteczna – 23.12.2026–3.01.2027 (dzień 9 z 12)
-Powód: przerwa świąteczna przewidziana w organizacji roku szkolnego – brak zajęć dydaktyczno-wychowawczych dla wszystkich klas.</t>
-  </si>
-  <si>
-    <t>Zimowa przerwa świąteczna – 23.12.2026–3.01.2027 (dzień 10 z 12)
-Powód: przerwa świąteczna przewidziana w organizacji roku szkolnego – brak zajęć dydaktyczno-wychowawczych dla wszystkich klas.</t>
-  </si>
-  <si>
-    <t>Zimowa przerwa świąteczna – 23.12.2026–3.01.2027 (dzień 11 z 12) · weekend
-Powód: przerwa świąteczna przewidziana w organizacji roku szkolnego – brak zajęć dydaktyczno-wychowawczych dla wszystkich klas.</t>
-  </si>
-  <si>
-    <t>Zimowa przerwa świąteczna – 23.12.2026–3.01.2027 (dzień 12 z 12) · weekend
-Powód: przerwa świąteczna przewidziana w organizacji roku szkolnego – brak zajęć dydaktyczno-wychowawczych dla wszystkich klas.</t>
-  </si>
-  <si>
-    <t>Ferie zimowe – 16.01.2027–31.01.2027 (dzień 1 z 16) · weekend
-Powód: ferie zimowe – brak zajęć dydaktyczno-wychowawczych dla wszystkich klas.</t>
-  </si>
-  <si>
-    <t>Ferie zimowe – 16.01.2027–31.01.2027 (dzień 2 z 16) · weekend
-Powód: ferie zimowe – brak zajęć dydaktyczno-wychowawczych dla wszystkich klas.</t>
-  </si>
-  <si>
-    <t>Ferie zimowe – 16.01.2027–31.01.2027 (dzień 3 z 16)
-Powód: ferie zimowe – brak zajęć dydaktyczno-wychowawczych dla wszystkich klas.</t>
-  </si>
-  <si>
-    <t>Ferie zimowe – 16.01.2027–31.01.2027 (dzień 4 z 16)
-Powód: ferie zimowe – brak zajęć dydaktyczno-wychowawczych dla wszystkich klas.</t>
-  </si>
-  <si>
-    <t>Ferie zimowe – 16.01.2027–31.01.2027 (dzień 5 z 16)
-Powód: ferie zimowe – brak zajęć dydaktyczno-wychowawczych dla wszystkich klas.</t>
-  </si>
-  <si>
-    <t>Ferie zimowe – 16.01.2027–31.01.2027 (dzień 6 z 16)
-Powód: ferie zimowe – brak zajęć dydaktyczno-wychowawczych dla wszystkich klas.
-Dodatkowo: EGZAMIN ZAWODOWY – sesja zimowa: ostatni dzień terminu głównego (5.01.2027 r. – 21.01.2027 r.).</t>
-  </si>
-  <si>
-    <t>Ferie zimowe – 16.01.2027–31.01.2027 (dzień 7 z 16)
-Powód: ferie zimowe – brak zajęć dydaktyczno-wychowawczych dla wszystkich klas.</t>
-  </si>
-  <si>
-    <t>Ferie zimowe – 16.01.2027–31.01.2027 (dzień 8 z 16) · weekend
-Powód: ferie zimowe – brak zajęć dydaktyczno-wychowawczych dla wszystkich klas.</t>
-  </si>
-  <si>
-    <t>Ferie zimowe – 16.01.2027–31.01.2027 (dzień 9 z 16) · weekend
-Powód: ferie zimowe – brak zajęć dydaktyczno-wychowawczych dla wszystkich klas.</t>
-  </si>
-  <si>
-    <t>Ferie zimowe – 16.01.2027–31.01.2027 (dzień 10 z 16)
-Powód: ferie zimowe – brak zajęć dydaktyczno-wychowawczych dla wszystkich klas.</t>
-  </si>
-  <si>
-    <t>Ferie zimowe – 16.01.2027–31.01.2027 (dzień 11 z 16)
-Powód: ferie zimowe – brak zajęć dydaktyczno-wychowawczych dla wszystkich klas.</t>
-  </si>
-  <si>
-    <t>Ferie zimowe – 16.01.2027–31.01.2027 (dzień 12 z 16)
-Powód: ferie zimowe – brak zajęć dydaktyczno-wychowawczych dla wszystkich klas.</t>
-  </si>
-  <si>
-    <t>Ferie zimowe – 16.01.2027–31.01.2027 (dzień 13 z 16)
-Powód: ferie zimowe – brak zajęć dydaktyczno-wychowawczych dla wszystkich klas.</t>
-  </si>
-  <si>
-    <t>Ferie zimowe – 16.01.2027–31.01.2027 (dzień 14 z 16)
-Powód: ferie zimowe – brak zajęć dydaktyczno-wychowawczych dla wszystkich klas.</t>
-  </si>
-  <si>
-    <t>Ferie zimowe – 16.01.2027–31.01.2027 (dzień 15 z 16) · weekend
-Powód: ferie zimowe – brak zajęć dydaktyczno-wychowawczych dla wszystkich klas.</t>
-  </si>
-  <si>
-    <t>Ferie zimowe – 16.01.2027–31.01.2027 (dzień 16 z 16) · weekend
-Powód: ferie zimowe – brak zajęć dydaktyczno-wychowawczych dla wszystkich klas.</t>
-  </si>
-  <si>
     <t>KLASY 4 TECHNIKUM: praktyki zawodowe – 2.02.2027–26.02.2027 (dzień 1 z 25)
 Powód: praktyka zawodowa u pracodawcy – klasy 4 Technikum nie mają zajęć w szkole; pozostałe klasy uczą się normalnie.</t>
   </si>
@@ -599,24 +465,158 @@
 Powód: wiosenna przerwa świąteczna (Wielkanoc 28.03, Poniedziałek Wielkanocny 29.03.2027) – brak zajęć dydaktyczno-wychowawczych.</t>
   </si>
   <si>
-    <t>Wiosenna przerwa świąteczna – 25.03.2027–30.03.2027 (dzień 4 z 6) · weekend
+    <t>Wiosenna przerwa świąteczna – 25.03.2027–30.03.2027 (dzień 6 z 6)
+Powód: wiosenna przerwa świąteczna (Wielkanoc 28.03, Poniedziałek Wielkanocny 29.03.2027) – brak zajęć dydaktyczno-wychowawczych.</t>
+  </si>
+  <si>
+    <t>nr tyg. kalendarz.</t>
+  </si>
+  <si>
+    <t>nr tyg. roku szk.</t>
+  </si>
+  <si>
+    <t>15:00 - RADA PEDAGOGICZNA:
+1) klasyfikacyjna: KLASY 5 TECHNIKUM oraz 3 SEMESTR BS II st.
+2) szkoleniowa: szkolenie z procedur egzaminu zawodowego</t>
+  </si>
+  <si>
+    <t>15:00 - RADA PEDAGOGICZNA:
+1) klasyfikacyjna: KLASY 1-4 TECHNIKUM, KLASY 1-3 BS I st., 1 SEMESTR BS II st.</t>
+  </si>
+  <si>
+    <t>15:00 - RADA PEDAGOGICZNA:
+1) plenarna: podsumowanie I półrocza</t>
+  </si>
+  <si>
+    <t>15:00 - RADA PEDAGOGICZNA:
+1) szkoleniowa</t>
+  </si>
+  <si>
+    <t>15:00 - RADA PEDAGOGICZNA:
+1) klasyfikacyjna: KLASY 5 TECHNIKUM oraz 4 SEMESTR BS II st.
+2) szkoleniowa: szkolenie z procedur egzaminu maturalnego</t>
+  </si>
+  <si>
+    <t>15:00 - RADA PEDAGOGICZNA:
+1) szkoleniowa: szkolenie z procedur egzaminów zawodowych</t>
+  </si>
+  <si>
+    <t>09:00 - RADA PEDAGOGICZNA: 31 sierpnia 2027 r.
+1) klasyfikacyjna: klasyfikacja uczniów po egzaminach poprawkowych
+2) plenarna: podsumowanie roku szkolnego 2026/2027
+3) inauguracyjna: rozpoczynająca rok szkolny 2027/2028</t>
+  </si>
+  <si>
+    <t>Wielkanoc (Niedziela Wielkanocna) - dzień ustawowo wolny
+Wiosenna przerwa świąteczna – 25.03.2027–30.03.2027 (dzień 4 z 6) · weekend
 Powód: wiosenna przerwa świąteczna (Wielkanoc 28.03, Poniedziałek Wielkanocny 29.03.2027) – brak zajęć dydaktyczno-wychowawczych.
 Dodatkowo: Wielkanoc.</t>
   </si>
   <si>
-    <t>Wiosenna przerwa świąteczna – 25.03.2027–30.03.2027 (dzień 5 z 6)
+    <t>Poniedziałek Wielkanocny - dzień ustawowo wolny
+Wiosenna przerwa świąteczna – 25.03.2027–30.03.2027 (dzień 5 z 6)
 Powód: wiosenna przerwa świąteczna (Wielkanoc 28.03, Poniedziałek Wielkanocny 29.03.2027) – brak zajęć dydaktyczno-wychowawczych.
 Dodatkowo: Poniedziałek Wielkanocny.</t>
   </si>
   <si>
-    <t>Wiosenna przerwa świąteczna – 25.03.2027–30.03.2027 (dzień 6 z 6)
-Powód: wiosenna przerwa świąteczna (Wielkanoc 28.03, Poniedziałek Wielkanocny 29.03.2027) – brak zajęć dydaktyczno-wychowawczych.</t>
-  </si>
-  <si>
-    <t>nr tyg. kalendarz.</t>
-  </si>
-  <si>
-    <t>nr tyg. roku szk.</t>
+    <t>Wniebowzięcie NMP / Święto Wojska Polskiego - dzień ustawowo wolny</t>
+  </si>
+  <si>
+    <t>Zimowa przerwa świąteczna – 23.12.2026–31.12.2026 (dzień 1 z 9)
+Powód: przerwa świąteczna przewidziana w organizacji roku szkolnego – brak zajęć dydaktyczno-wychowawczych dla wszystkich klas.</t>
+  </si>
+  <si>
+    <t>Zimowa przerwa świąteczna – 23.12.2026–31.12.2026 (dzień 2 z 9)
+Powód: przerwa świąteczna przewidziana w organizacji roku szkolnego – brak zajęć dydaktyczno-wychowawczych dla wszystkich klas.</t>
+  </si>
+  <si>
+    <t>Boże Narodzenie (pierwszy dzień) - dzień ustawowo wolny
+Zimowa przerwa świąteczna – 23.12.2026–31.12.2026 (dzień 3 z 9)
+Powód: przerwa świąteczna przewidziana w organizacji roku szkolnego – brak zajęć dydaktyczno-wychowawczych dla wszystkich klas.</t>
+  </si>
+  <si>
+    <t>Boże Narodzenie (drugi dzień) - dzień ustawowo wolny
+Zimowa przerwa świąteczna – 23.12.2026–31.12.2026 (dzień 4 z 9) · weekend
+Powód: przerwa świąteczna przewidziana w organizacji roku szkolnego – brak zajęć dydaktyczno-wychowawczych dla wszystkich klas.</t>
+  </si>
+  <si>
+    <t>Zimowa przerwa świąteczna – 23.12.2026–31.12.2026 (dzień 5 z 9) · weekend
+Powód: przerwa świąteczna przewidziana w organizacji roku szkolnego – brak zajęć dydaktyczno-wychowawczych dla wszystkich klas.</t>
+  </si>
+  <si>
+    <t>Zimowa przerwa świąteczna – 23.12.2026–31.12.2026 (dzień 6 z 9)
+Powód: przerwa świąteczna przewidziana w organizacji roku szkolnego – brak zajęć dydaktyczno-wychowawczych dla wszystkich klas.</t>
+  </si>
+  <si>
+    <t>Zimowa przerwa świąteczna – 23.12.2026–31.12.2026 (dzień 7 z 9)
+Powód: przerwa świąteczna przewidziana w organizacji roku szkolnego – brak zajęć dydaktyczno-wychowawczych dla wszystkich klas.</t>
+  </si>
+  <si>
+    <t>Zimowa przerwa świąteczna – 23.12.2026–31.12.2026 (dzień 8 z 9)
+Powód: przerwa świąteczna przewidziana w organizacji roku szkolnego – brak zajęć dydaktyczno-wychowawczych dla wszystkich klas.</t>
+  </si>
+  <si>
+    <t>Zimowa przerwa świąteczna – 23.12.2026–31.12.2026 (dzień 9 z 9)
+Powód: przerwa świąteczna przewidziana w organizacji roku szkolnego – brak zajęć dydaktyczno-wychowawczych dla wszystkich klas.</t>
+  </si>
+  <si>
+    <t>Nowy Rok - dzień ustawowo wolny</t>
+  </si>
+  <si>
+    <t>Ferie zimowe – 18.01.2027–31.01.2027 (dzień 1 z 14)
+Powód: ferie zimowe (tura: podkarpackie, podlaskie, dolnośląskie, łódzkie, śląskie, opolskie) – brak zajęć dydaktyczno-wychowawczych dla wszystkich klas.</t>
+  </si>
+  <si>
+    <t>Ferie zimowe – 18.01.2027–31.01.2027 (dzień 2 z 14)
+Powód: ferie zimowe (tura: podkarpackie, podlaskie, dolnośląskie, łódzkie, śląskie, opolskie) – brak zajęć dydaktyczno-wychowawczych dla wszystkich klas.</t>
+  </si>
+  <si>
+    <t>Ferie zimowe – 18.01.2027–31.01.2027 (dzień 3 z 14)
+Powód: ferie zimowe (tura: podkarpackie, podlaskie, dolnośląskie, łódzkie, śląskie, opolskie) – brak zajęć dydaktyczno-wychowawczych dla wszystkich klas.</t>
+  </si>
+  <si>
+    <t>Ferie zimowe – 18.01.2027–31.01.2027 (dzień 4 z 14)
+Powód: ferie zimowe (tura: podkarpackie, podlaskie, dolnośląskie, łódzkie, śląskie, opolskie) – brak zajęć dydaktyczno-wychowawczych dla wszystkich klas.</t>
+  </si>
+  <si>
+    <t>Ferie zimowe – 18.01.2027–31.01.2027 (dzień 5 z 14)
+Powód: ferie zimowe (tura: podkarpackie, podlaskie, dolnośląskie, łódzkie, śląskie, opolskie) – brak zajęć dydaktyczno-wychowawczych dla wszystkich klas.</t>
+  </si>
+  <si>
+    <t>Ferie zimowe – 18.01.2027–31.01.2027 (dzień 6 z 14) · weekend
+Powód: ferie zimowe (tura: podkarpackie, podlaskie, dolnośląskie, łódzkie, śląskie, opolskie) – brak zajęć dydaktyczno-wychowawczych dla wszystkich klas.</t>
+  </si>
+  <si>
+    <t>Ferie zimowe – 18.01.2027–31.01.2027 (dzień 7 z 14) · weekend
+Powód: ferie zimowe (tura: podkarpackie, podlaskie, dolnośląskie, łódzkie, śląskie, opolskie) – brak zajęć dydaktyczno-wychowawczych dla wszystkich klas.</t>
+  </si>
+  <si>
+    <t>Ferie zimowe – 18.01.2027–31.01.2027 (dzień 8 z 14)
+Powód: ferie zimowe (tura: podkarpackie, podlaskie, dolnośląskie, łódzkie, śląskie, opolskie) – brak zajęć dydaktyczno-wychowawczych dla wszystkich klas.</t>
+  </si>
+  <si>
+    <t>Ferie zimowe – 18.01.2027–31.01.2027 (dzień 9 z 14)
+Powód: ferie zimowe (tura: podkarpackie, podlaskie, dolnośląskie, łódzkie, śląskie, opolskie) – brak zajęć dydaktyczno-wychowawczych dla wszystkich klas.</t>
+  </si>
+  <si>
+    <t>Ferie zimowe – 18.01.2027–31.01.2027 (dzień 10 z 14)
+Powód: ferie zimowe (tura: podkarpackie, podlaskie, dolnośląskie, łódzkie, śląskie, opolskie) – brak zajęć dydaktyczno-wychowawczych dla wszystkich klas.</t>
+  </si>
+  <si>
+    <t>Ferie zimowe – 18.01.2027–31.01.2027 (dzień 11 z 14)
+Powód: ferie zimowe (tura: podkarpackie, podlaskie, dolnośląskie, łódzkie, śląskie, opolskie) – brak zajęć dydaktyczno-wychowawczych dla wszystkich klas.</t>
+  </si>
+  <si>
+    <t>Ferie zimowe – 18.01.2027–31.01.2027 (dzień 12 z 14)
+Powód: ferie zimowe (tura: podkarpackie, podlaskie, dolnośląskie, łódzkie, śląskie, opolskie) – brak zajęć dydaktyczno-wychowawczych dla wszystkich klas.</t>
+  </si>
+  <si>
+    <t>Ferie zimowe – 18.01.2027–31.01.2027 (dzień 13 z 14) · weekend
+Powód: ferie zimowe (tura: podkarpackie, podlaskie, dolnośląskie, łódzkie, śląskie, opolskie) – brak zajęć dydaktyczno-wychowawczych dla wszystkich klas.</t>
+  </si>
+  <si>
+    <t>Ferie zimowe – 18.01.2027–31.01.2027 (dzień 14 z 14) · weekend
+Powód: ferie zimowe (tura: podkarpackie, podlaskie, dolnośląskie, łódzkie, śląskie, opolskie) – brak zajęć dydaktyczno-wychowawczych dla wszystkich klas.</t>
   </si>
 </sst>
 </file>
@@ -682,7 +682,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -701,6 +701,9 @@
     </xf>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1048,7 +1051,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>160</v>
+        <v>123</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>1</v>
@@ -1066,7 +1069,7 @@
         <v>5</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>161</v>
+        <v>124</v>
       </c>
     </row>
     <row r="2" spans="1:8" ht="48" x14ac:dyDescent="0.2">
@@ -1087,7 +1090,7 @@
       <c r="F2" s="3"/>
       <c r="G2" s="3"/>
       <c r="H2" s="6">
-        <f>IF(A2&gt;DATE(2027,6,26),"",INT((A2-DATE(2026,8,31))/7)+1)</f>
+        <f>IF(A2&gt;DATE(2027,6,25),"",INT((A2-DATE(2026,8,31))/7)+1)</f>
         <v>1</v>
       </c>
     </row>
@@ -1103,10 +1106,11 @@
         <v>7</v>
       </c>
       <c r="D3" s="3"/>
+      <c r="E3" s="7"/>
       <c r="F3" s="3"/>
       <c r="G3" s="3"/>
       <c r="H3" s="6">
-        <f t="shared" ref="H3:H66" si="1">IF(A3&gt;DATE(2027,6,26),"",INT((A3-DATE(2026,8,31))/7)+1)</f>
+        <f t="shared" ref="H3:H66" si="1">IF(A3&gt;DATE(2027,6,25),"",INT((A3-DATE(2026,8,31))/7)+1)</f>
         <v>1</v>
       </c>
     </row>
@@ -1250,7 +1254,7 @@
         <v>34</v>
       </c>
       <c r="F10" s="3" t="s">
-        <v>71</v>
+        <v>64</v>
       </c>
       <c r="G10" s="3"/>
       <c r="H10" s="6">
@@ -1270,6 +1274,7 @@
         <v>8</v>
       </c>
       <c r="D11" s="3"/>
+      <c r="E11" s="7"/>
       <c r="F11" s="3"/>
       <c r="G11" s="3"/>
       <c r="H11" s="6">
@@ -1771,7 +1776,7 @@
         <v>12</v>
       </c>
       <c r="D36" s="3" t="s">
-        <v>75</v>
+        <v>68</v>
       </c>
       <c r="E36" s="3"/>
       <c r="F36" s="3"/>
@@ -1793,7 +1798,7 @@
         <v>6</v>
       </c>
       <c r="D37" s="3" t="s">
-        <v>76</v>
+        <v>69</v>
       </c>
       <c r="E37" s="3"/>
       <c r="F37" s="3"/>
@@ -1815,7 +1820,7 @@
         <v>7</v>
       </c>
       <c r="D38" s="3" t="s">
-        <v>77</v>
+        <v>70</v>
       </c>
       <c r="E38" s="3"/>
       <c r="F38" s="3"/>
@@ -1837,7 +1842,7 @@
         <v>8</v>
       </c>
       <c r="D39" s="3" t="s">
-        <v>78</v>
+        <v>71</v>
       </c>
       <c r="E39" s="3"/>
       <c r="F39" s="3"/>
@@ -1859,7 +1864,7 @@
         <v>9</v>
       </c>
       <c r="D40" s="3" t="s">
-        <v>79</v>
+        <v>72</v>
       </c>
       <c r="E40" s="3"/>
       <c r="F40" s="3"/>
@@ -1881,7 +1886,7 @@
         <v>10</v>
       </c>
       <c r="D41" s="3" t="s">
-        <v>80</v>
+        <v>73</v>
       </c>
       <c r="E41" s="3"/>
       <c r="F41" s="3"/>
@@ -1903,7 +1908,7 @@
         <v>11</v>
       </c>
       <c r="D42" s="3" t="s">
-        <v>81</v>
+        <v>74</v>
       </c>
       <c r="E42" s="3"/>
       <c r="F42" s="3"/>
@@ -1925,7 +1930,7 @@
         <v>12</v>
       </c>
       <c r="D43" s="3" t="s">
-        <v>82</v>
+        <v>75</v>
       </c>
       <c r="E43" s="3"/>
       <c r="F43" s="3"/>
@@ -1947,7 +1952,7 @@
         <v>6</v>
       </c>
       <c r="D44" s="3" t="s">
-        <v>83</v>
+        <v>76</v>
       </c>
       <c r="E44" s="3"/>
       <c r="F44" s="3"/>
@@ -1969,7 +1974,7 @@
         <v>7</v>
       </c>
       <c r="D45" s="3" t="s">
-        <v>84</v>
+        <v>77</v>
       </c>
       <c r="E45" s="3"/>
       <c r="F45" s="3"/>
@@ -1991,7 +1996,7 @@
         <v>8</v>
       </c>
       <c r="D46" s="3" t="s">
-        <v>85</v>
+        <v>78</v>
       </c>
       <c r="E46" s="3"/>
       <c r="F46" s="3"/>
@@ -2013,7 +2018,7 @@
         <v>9</v>
       </c>
       <c r="D47" s="3" t="s">
-        <v>86</v>
+        <v>79</v>
       </c>
       <c r="E47" s="3"/>
       <c r="F47" s="3"/>
@@ -2035,7 +2040,7 @@
         <v>10</v>
       </c>
       <c r="D48" s="3" t="s">
-        <v>87</v>
+        <v>80</v>
       </c>
       <c r="E48" s="3"/>
       <c r="F48" s="3"/>
@@ -2057,7 +2062,7 @@
         <v>11</v>
       </c>
       <c r="D49" s="3" t="s">
-        <v>88</v>
+        <v>81</v>
       </c>
       <c r="E49" s="3"/>
       <c r="F49" s="3"/>
@@ -2079,7 +2084,7 @@
         <v>12</v>
       </c>
       <c r="D50" s="3" t="s">
-        <v>89</v>
+        <v>82</v>
       </c>
       <c r="E50" s="3"/>
       <c r="F50" s="3"/>
@@ -2101,7 +2106,7 @@
         <v>6</v>
       </c>
       <c r="D51" s="3" t="s">
-        <v>90</v>
+        <v>83</v>
       </c>
       <c r="E51" s="3"/>
       <c r="F51" s="3"/>
@@ -2123,7 +2128,7 @@
         <v>7</v>
       </c>
       <c r="D52" s="3" t="s">
-        <v>91</v>
+        <v>84</v>
       </c>
       <c r="E52" s="3"/>
       <c r="F52" s="3"/>
@@ -2145,7 +2150,7 @@
         <v>8</v>
       </c>
       <c r="D53" s="3" t="s">
-        <v>92</v>
+        <v>85</v>
       </c>
       <c r="E53" s="3"/>
       <c r="F53" s="3"/>
@@ -2167,7 +2172,7 @@
         <v>9</v>
       </c>
       <c r="D54" s="3" t="s">
-        <v>93</v>
+        <v>86</v>
       </c>
       <c r="E54" s="3"/>
       <c r="F54" s="3"/>
@@ -2189,7 +2194,7 @@
         <v>10</v>
       </c>
       <c r="D55" s="3" t="s">
-        <v>94</v>
+        <v>87</v>
       </c>
       <c r="E55" s="3"/>
       <c r="F55" s="3"/>
@@ -2211,7 +2216,7 @@
         <v>11</v>
       </c>
       <c r="D56" s="3" t="s">
-        <v>95</v>
+        <v>88</v>
       </c>
       <c r="E56" s="3"/>
       <c r="F56" s="3"/>
@@ -2233,7 +2238,7 @@
         <v>12</v>
       </c>
       <c r="D57" s="3" t="s">
-        <v>96</v>
+        <v>89</v>
       </c>
       <c r="E57" s="3"/>
       <c r="F57" s="3"/>
@@ -2255,7 +2260,7 @@
         <v>6</v>
       </c>
       <c r="D58" s="3" t="s">
-        <v>97</v>
+        <v>90</v>
       </c>
       <c r="E58" s="3"/>
       <c r="F58" s="3"/>
@@ -2277,7 +2282,7 @@
         <v>7</v>
       </c>
       <c r="D59" s="3" t="s">
-        <v>98</v>
+        <v>91</v>
       </c>
       <c r="E59" s="3"/>
       <c r="F59" s="3"/>
@@ -2299,7 +2304,7 @@
         <v>8</v>
       </c>
       <c r="D60" s="3" t="s">
-        <v>99</v>
+        <v>92</v>
       </c>
       <c r="E60" s="3"/>
       <c r="F60" s="3"/>
@@ -2321,7 +2326,7 @@
         <v>9</v>
       </c>
       <c r="D61" s="3" t="s">
-        <v>100</v>
+        <v>93</v>
       </c>
       <c r="E61" s="3" t="s">
         <v>35</v>
@@ -2451,7 +2456,7 @@
       <c r="F67" s="3"/>
       <c r="G67" s="3"/>
       <c r="H67" s="6">
-        <f t="shared" ref="H67:H130" si="3">IF(A67&gt;DATE(2027,6,26),"",INT((A67-DATE(2026,8,31))/7)+1)</f>
+        <f t="shared" ref="H67:H130" si="3">IF(A67&gt;DATE(2027,6,25),"",INT((A67-DATE(2026,8,31))/7)+1)</f>
         <v>10</v>
       </c>
     </row>
@@ -3127,7 +3132,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="101" spans="1:8" ht="64" x14ac:dyDescent="0.2">
+    <row r="101" spans="1:8" ht="80" x14ac:dyDescent="0.2">
       <c r="A101" s="2">
         <v>46365</v>
       </c>
@@ -3141,7 +3146,7 @@
       <c r="D101" s="3"/>
       <c r="E101" s="3"/>
       <c r="F101" s="3" t="s">
-        <v>40</v>
+        <v>125</v>
       </c>
       <c r="G101" s="3"/>
       <c r="H101" s="6">
@@ -3181,10 +3186,10 @@
         <v>9</v>
       </c>
       <c r="D103" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="E103" s="3" t="s">
         <v>41</v>
-      </c>
-      <c r="E103" s="3" t="s">
-        <v>42</v>
       </c>
       <c r="F103" s="3"/>
       <c r="G103" s="3"/>
@@ -3425,7 +3430,7 @@
         <v>7</v>
       </c>
       <c r="D115" s="3" t="s">
-        <v>101</v>
+        <v>135</v>
       </c>
       <c r="E115" s="3"/>
       <c r="F115" s="3"/>
@@ -3447,7 +3452,7 @@
         <v>8</v>
       </c>
       <c r="D116" s="3" t="s">
-        <v>102</v>
+        <v>136</v>
       </c>
       <c r="E116" s="3"/>
       <c r="F116" s="3"/>
@@ -3457,7 +3462,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="117" spans="1:8" ht="80" x14ac:dyDescent="0.2">
+    <row r="117" spans="1:8" ht="112" x14ac:dyDescent="0.2">
       <c r="A117" s="2">
         <v>46381</v>
       </c>
@@ -3469,7 +3474,7 @@
         <v>9</v>
       </c>
       <c r="D117" s="3" t="s">
-        <v>103</v>
+        <v>137</v>
       </c>
       <c r="E117" s="3"/>
       <c r="F117" s="3"/>
@@ -3479,7 +3484,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="118" spans="1:8" ht="80" x14ac:dyDescent="0.2">
+    <row r="118" spans="1:8" ht="112" x14ac:dyDescent="0.2">
       <c r="A118" s="2">
         <v>46382</v>
       </c>
@@ -3491,7 +3496,7 @@
         <v>10</v>
       </c>
       <c r="D118" s="3" t="s">
-        <v>104</v>
+        <v>138</v>
       </c>
       <c r="E118" s="3"/>
       <c r="F118" s="3"/>
@@ -3513,7 +3518,7 @@
         <v>11</v>
       </c>
       <c r="D119" s="3" t="s">
-        <v>105</v>
+        <v>139</v>
       </c>
       <c r="E119" s="3"/>
       <c r="F119" s="3"/>
@@ -3535,7 +3540,7 @@
         <v>12</v>
       </c>
       <c r="D120" s="3" t="s">
-        <v>106</v>
+        <v>140</v>
       </c>
       <c r="E120" s="3"/>
       <c r="F120" s="3"/>
@@ -3557,7 +3562,7 @@
         <v>6</v>
       </c>
       <c r="D121" s="3" t="s">
-        <v>107</v>
+        <v>141</v>
       </c>
       <c r="E121" s="3"/>
       <c r="F121" s="3"/>
@@ -3579,7 +3584,7 @@
         <v>7</v>
       </c>
       <c r="D122" s="3" t="s">
-        <v>108</v>
+        <v>142</v>
       </c>
       <c r="E122" s="3"/>
       <c r="F122" s="3"/>
@@ -3601,7 +3606,7 @@
         <v>8</v>
       </c>
       <c r="D123" s="3" t="s">
-        <v>109</v>
+        <v>143</v>
       </c>
       <c r="E123" s="3"/>
       <c r="F123" s="3"/>
@@ -3611,7 +3616,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="124" spans="1:8" ht="80" x14ac:dyDescent="0.2">
+    <row r="124" spans="1:8" ht="16" x14ac:dyDescent="0.2">
       <c r="A124" s="2">
         <v>46388</v>
       </c>
@@ -3623,7 +3628,7 @@
         <v>9</v>
       </c>
       <c r="D124" s="3" t="s">
-        <v>110</v>
+        <v>144</v>
       </c>
       <c r="E124" s="3"/>
       <c r="F124" s="3"/>
@@ -3633,7 +3638,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="125" spans="1:8" ht="80" x14ac:dyDescent="0.2">
+    <row r="125" spans="1:8" ht="16" x14ac:dyDescent="0.2">
       <c r="A125" s="2">
         <v>46389</v>
       </c>
@@ -3644,9 +3649,7 @@
       <c r="C125" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="D125" s="3" t="s">
-        <v>111</v>
-      </c>
+      <c r="D125" s="3"/>
       <c r="E125" s="3"/>
       <c r="F125" s="3"/>
       <c r="G125" s="3"/>
@@ -3655,7 +3658,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="126" spans="1:8" ht="80" x14ac:dyDescent="0.2">
+    <row r="126" spans="1:8" ht="16" x14ac:dyDescent="0.2">
       <c r="A126" s="2">
         <v>46390</v>
       </c>
@@ -3666,9 +3669,7 @@
       <c r="C126" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="D126" s="3" t="s">
-        <v>112</v>
-      </c>
+      <c r="D126" s="3"/>
       <c r="E126" s="3"/>
       <c r="F126" s="3"/>
       <c r="G126" s="3"/>
@@ -3691,7 +3692,7 @@
       <c r="D127" s="3"/>
       <c r="E127" s="3"/>
       <c r="F127" s="3" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="G127" s="3"/>
       <c r="H127" s="6">
@@ -3711,7 +3712,7 @@
         <v>6</v>
       </c>
       <c r="D128" s="3" t="s">
-        <v>72</v>
+        <v>65</v>
       </c>
       <c r="E128" s="3"/>
       <c r="F128" s="3"/>
@@ -3755,7 +3756,7 @@
         <v>8</v>
       </c>
       <c r="D130" s="3" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="E130" s="3"/>
       <c r="F130" s="3"/>
@@ -3781,7 +3782,7 @@
       <c r="F131" s="3"/>
       <c r="G131" s="3"/>
       <c r="H131" s="6">
-        <f t="shared" ref="H131:H194" si="5">IF(A131&gt;DATE(2027,6,26),"",INT((A131-DATE(2026,8,31))/7)+1)</f>
+        <f t="shared" ref="H131:H194" si="5">IF(A131&gt;DATE(2027,6,25),"",INT((A131-DATE(2026,8,31))/7)+1)</f>
         <v>19</v>
       </c>
     </row>
@@ -3838,7 +3839,7 @@
       </c>
       <c r="D134" s="3"/>
       <c r="E134" s="3" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="F134" s="3"/>
       <c r="G134" s="3"/>
@@ -3860,7 +3861,7 @@
       </c>
       <c r="D135" s="4"/>
       <c r="E135" s="3" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="F135" s="3"/>
       <c r="G135" s="3"/>
@@ -3883,7 +3884,7 @@
       <c r="D136" s="3"/>
       <c r="E136" s="3"/>
       <c r="F136" s="3" t="s">
-        <v>47</v>
+        <v>126</v>
       </c>
       <c r="G136" s="3"/>
       <c r="H136" s="6">
@@ -3924,7 +3925,7 @@
       </c>
       <c r="D138" s="3"/>
       <c r="E138" s="3" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="F138" s="3"/>
       <c r="G138" s="3"/>
@@ -3933,7 +3934,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="139" spans="1:8" ht="64" x14ac:dyDescent="0.2">
+    <row r="139" spans="1:8" ht="16" x14ac:dyDescent="0.2">
       <c r="A139" s="2">
         <v>46403</v>
       </c>
@@ -3944,9 +3945,7 @@
       <c r="C139" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="D139" s="3" t="s">
-        <v>113</v>
-      </c>
+      <c r="D139" s="3"/>
       <c r="E139" s="3"/>
       <c r="F139" s="3"/>
       <c r="G139" s="3"/>
@@ -3955,7 +3954,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="140" spans="1:8" ht="64" x14ac:dyDescent="0.2">
+    <row r="140" spans="1:8" ht="16" x14ac:dyDescent="0.2">
       <c r="A140" s="2">
         <v>46404</v>
       </c>
@@ -3966,9 +3965,7 @@
       <c r="C140" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="D140" s="3" t="s">
-        <v>114</v>
-      </c>
+      <c r="D140" s="3"/>
       <c r="E140" s="3"/>
       <c r="F140" s="3"/>
       <c r="G140" s="3"/>
@@ -3977,7 +3974,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="141" spans="1:8" ht="64" x14ac:dyDescent="0.2">
+    <row r="141" spans="1:8" ht="80" x14ac:dyDescent="0.2">
       <c r="A141" s="2">
         <v>46405</v>
       </c>
@@ -3989,7 +3986,7 @@
         <v>12</v>
       </c>
       <c r="D141" s="3" t="s">
-        <v>115</v>
+        <v>145</v>
       </c>
       <c r="E141" s="3"/>
       <c r="F141" s="3"/>
@@ -3999,7 +3996,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="142" spans="1:8" ht="64" x14ac:dyDescent="0.2">
+    <row r="142" spans="1:8" ht="80" x14ac:dyDescent="0.2">
       <c r="A142" s="2">
         <v>46406</v>
       </c>
@@ -4011,7 +4008,7 @@
         <v>6</v>
       </c>
       <c r="D142" s="3" t="s">
-        <v>116</v>
+        <v>146</v>
       </c>
       <c r="E142" s="3"/>
       <c r="F142" s="3"/>
@@ -4021,7 +4018,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="143" spans="1:8" ht="64" x14ac:dyDescent="0.2">
+    <row r="143" spans="1:8" ht="80" x14ac:dyDescent="0.2">
       <c r="A143" s="2">
         <v>46407</v>
       </c>
@@ -4033,7 +4030,7 @@
         <v>7</v>
       </c>
       <c r="D143" s="3" t="s">
-        <v>117</v>
+        <v>147</v>
       </c>
       <c r="E143" s="3"/>
       <c r="F143" s="3"/>
@@ -4043,7 +4040,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="144" spans="1:8" ht="112" x14ac:dyDescent="0.2">
+    <row r="144" spans="1:8" ht="80" x14ac:dyDescent="0.2">
       <c r="A144" s="2">
         <v>46408</v>
       </c>
@@ -4055,7 +4052,7 @@
         <v>8</v>
       </c>
       <c r="D144" s="3" t="s">
-        <v>118</v>
+        <v>148</v>
       </c>
       <c r="E144" s="3"/>
       <c r="F144" s="3"/>
@@ -4065,7 +4062,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="145" spans="1:8" ht="64" x14ac:dyDescent="0.2">
+    <row r="145" spans="1:8" ht="80" x14ac:dyDescent="0.2">
       <c r="A145" s="2">
         <v>46409</v>
       </c>
@@ -4077,7 +4074,7 @@
         <v>9</v>
       </c>
       <c r="D145" s="3" t="s">
-        <v>119</v>
+        <v>149</v>
       </c>
       <c r="E145" s="3"/>
       <c r="F145" s="3"/>
@@ -4087,7 +4084,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="146" spans="1:8" ht="64" x14ac:dyDescent="0.2">
+    <row r="146" spans="1:8" ht="80" x14ac:dyDescent="0.2">
       <c r="A146" s="2">
         <v>46410</v>
       </c>
@@ -4099,7 +4096,7 @@
         <v>10</v>
       </c>
       <c r="D146" s="3" t="s">
-        <v>120</v>
+        <v>150</v>
       </c>
       <c r="E146" s="3"/>
       <c r="F146" s="3"/>
@@ -4109,7 +4106,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="147" spans="1:8" ht="64" x14ac:dyDescent="0.2">
+    <row r="147" spans="1:8" ht="80" x14ac:dyDescent="0.2">
       <c r="A147" s="2">
         <v>46411</v>
       </c>
@@ -4121,7 +4118,7 @@
         <v>11</v>
       </c>
       <c r="D147" s="3" t="s">
-        <v>121</v>
+        <v>151</v>
       </c>
       <c r="E147" s="3"/>
       <c r="F147" s="3"/>
@@ -4131,7 +4128,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="148" spans="1:8" ht="64" x14ac:dyDescent="0.2">
+    <row r="148" spans="1:8" ht="80" x14ac:dyDescent="0.2">
       <c r="A148" s="2">
         <v>46412</v>
       </c>
@@ -4143,7 +4140,7 @@
         <v>12</v>
       </c>
       <c r="D148" s="3" t="s">
-        <v>122</v>
+        <v>152</v>
       </c>
       <c r="E148" s="3"/>
       <c r="F148" s="3"/>
@@ -4153,7 +4150,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="149" spans="1:8" ht="64" x14ac:dyDescent="0.2">
+    <row r="149" spans="1:8" ht="80" x14ac:dyDescent="0.2">
       <c r="A149" s="2">
         <v>46413</v>
       </c>
@@ -4165,7 +4162,7 @@
         <v>6</v>
       </c>
       <c r="D149" s="3" t="s">
-        <v>123</v>
+        <v>153</v>
       </c>
       <c r="E149" s="3"/>
       <c r="F149" s="3"/>
@@ -4175,7 +4172,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="150" spans="1:8" ht="64" x14ac:dyDescent="0.2">
+    <row r="150" spans="1:8" ht="80" x14ac:dyDescent="0.2">
       <c r="A150" s="2">
         <v>46414</v>
       </c>
@@ -4187,7 +4184,7 @@
         <v>7</v>
       </c>
       <c r="D150" s="3" t="s">
-        <v>124</v>
+        <v>154</v>
       </c>
       <c r="E150" s="3"/>
       <c r="F150" s="3"/>
@@ -4197,7 +4194,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="151" spans="1:8" ht="64" x14ac:dyDescent="0.2">
+    <row r="151" spans="1:8" ht="80" x14ac:dyDescent="0.2">
       <c r="A151" s="2">
         <v>46415</v>
       </c>
@@ -4209,7 +4206,7 @@
         <v>8</v>
       </c>
       <c r="D151" s="3" t="s">
-        <v>125</v>
+        <v>155</v>
       </c>
       <c r="E151" s="3"/>
       <c r="F151" s="3"/>
@@ -4219,7 +4216,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="152" spans="1:8" ht="64" x14ac:dyDescent="0.2">
+    <row r="152" spans="1:8" ht="80" x14ac:dyDescent="0.2">
       <c r="A152" s="2">
         <v>46416</v>
       </c>
@@ -4231,7 +4228,7 @@
         <v>9</v>
       </c>
       <c r="D152" s="3" t="s">
-        <v>126</v>
+        <v>156</v>
       </c>
       <c r="E152" s="3"/>
       <c r="F152" s="3"/>
@@ -4241,7 +4238,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="153" spans="1:8" ht="64" x14ac:dyDescent="0.2">
+    <row r="153" spans="1:8" ht="80" x14ac:dyDescent="0.2">
       <c r="A153" s="2">
         <v>46417</v>
       </c>
@@ -4253,7 +4250,7 @@
         <v>10</v>
       </c>
       <c r="D153" s="3" t="s">
-        <v>127</v>
+        <v>157</v>
       </c>
       <c r="E153" s="3"/>
       <c r="F153" s="3"/>
@@ -4263,7 +4260,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="154" spans="1:8" ht="64" x14ac:dyDescent="0.2">
+    <row r="154" spans="1:8" ht="80" x14ac:dyDescent="0.2">
       <c r="A154" s="2">
         <v>46418</v>
       </c>
@@ -4275,7 +4272,7 @@
         <v>11</v>
       </c>
       <c r="D154" s="3" t="s">
-        <v>128</v>
+        <v>158</v>
       </c>
       <c r="E154" s="3"/>
       <c r="F154" s="3"/>
@@ -4319,7 +4316,7 @@
         <v>6</v>
       </c>
       <c r="D156" s="3" t="s">
-        <v>129</v>
+        <v>94</v>
       </c>
       <c r="E156" s="3"/>
       <c r="F156" s="3"/>
@@ -4341,11 +4338,11 @@
         <v>7</v>
       </c>
       <c r="D157" s="3" t="s">
-        <v>130</v>
+        <v>95</v>
       </c>
       <c r="E157" s="3"/>
       <c r="F157" s="3" t="s">
-        <v>49</v>
+        <v>127</v>
       </c>
       <c r="G157" s="3"/>
       <c r="H157" s="6">
@@ -4365,7 +4362,7 @@
         <v>8</v>
       </c>
       <c r="D158" s="3" t="s">
-        <v>131</v>
+        <v>96</v>
       </c>
       <c r="E158" s="3"/>
       <c r="F158" s="3"/>
@@ -4387,7 +4384,7 @@
         <v>9</v>
       </c>
       <c r="D159" s="3" t="s">
-        <v>132</v>
+        <v>97</v>
       </c>
       <c r="E159" s="3"/>
       <c r="F159" s="3"/>
@@ -4409,7 +4406,7 @@
         <v>10</v>
       </c>
       <c r="D160" s="3" t="s">
-        <v>133</v>
+        <v>98</v>
       </c>
       <c r="E160" s="3"/>
       <c r="F160" s="3"/>
@@ -4431,7 +4428,7 @@
         <v>11</v>
       </c>
       <c r="D161" s="3" t="s">
-        <v>134</v>
+        <v>99</v>
       </c>
       <c r="E161" s="3"/>
       <c r="F161" s="3"/>
@@ -4453,7 +4450,7 @@
         <v>12</v>
       </c>
       <c r="D162" s="3" t="s">
-        <v>135</v>
+        <v>100</v>
       </c>
       <c r="E162" s="3"/>
       <c r="F162" s="3"/>
@@ -4475,7 +4472,7 @@
         <v>6</v>
       </c>
       <c r="D163" s="3" t="s">
-        <v>136</v>
+        <v>101</v>
       </c>
       <c r="E163" s="3"/>
       <c r="F163" s="3"/>
@@ -4497,7 +4494,7 @@
         <v>7</v>
       </c>
       <c r="D164" s="3" t="s">
-        <v>137</v>
+        <v>102</v>
       </c>
       <c r="E164" s="3"/>
       <c r="F164" s="3"/>
@@ -4519,7 +4516,7 @@
         <v>8</v>
       </c>
       <c r="D165" s="3" t="s">
-        <v>138</v>
+        <v>103</v>
       </c>
       <c r="E165" s="3"/>
       <c r="F165" s="3"/>
@@ -4541,7 +4538,7 @@
         <v>9</v>
       </c>
       <c r="D166" s="3" t="s">
-        <v>139</v>
+        <v>104</v>
       </c>
       <c r="E166" s="3"/>
       <c r="F166" s="3"/>
@@ -4563,7 +4560,7 @@
         <v>10</v>
       </c>
       <c r="D167" s="3" t="s">
-        <v>140</v>
+        <v>105</v>
       </c>
       <c r="E167" s="3"/>
       <c r="F167" s="3"/>
@@ -4585,7 +4582,7 @@
         <v>11</v>
       </c>
       <c r="D168" s="3" t="s">
-        <v>141</v>
+        <v>106</v>
       </c>
       <c r="E168" s="3"/>
       <c r="F168" s="3"/>
@@ -4607,7 +4604,7 @@
         <v>12</v>
       </c>
       <c r="D169" s="3" t="s">
-        <v>142</v>
+        <v>107</v>
       </c>
       <c r="E169" s="3"/>
       <c r="F169" s="3"/>
@@ -4629,7 +4626,7 @@
         <v>6</v>
       </c>
       <c r="D170" s="3" t="s">
-        <v>143</v>
+        <v>108</v>
       </c>
       <c r="E170" s="3"/>
       <c r="F170" s="3"/>
@@ -4651,7 +4648,7 @@
         <v>7</v>
       </c>
       <c r="D171" s="3" t="s">
-        <v>144</v>
+        <v>109</v>
       </c>
       <c r="E171" s="3"/>
       <c r="F171" s="3"/>
@@ -4673,7 +4670,7 @@
         <v>8</v>
       </c>
       <c r="D172" s="3" t="s">
-        <v>145</v>
+        <v>110</v>
       </c>
       <c r="E172" s="3"/>
       <c r="F172" s="3"/>
@@ -4695,7 +4692,7 @@
         <v>9</v>
       </c>
       <c r="D173" s="3" t="s">
-        <v>146</v>
+        <v>111</v>
       </c>
       <c r="E173" s="3"/>
       <c r="F173" s="3"/>
@@ -4717,7 +4714,7 @@
         <v>10</v>
       </c>
       <c r="D174" s="3" t="s">
-        <v>147</v>
+        <v>112</v>
       </c>
       <c r="E174" s="3"/>
       <c r="F174" s="3"/>
@@ -4739,7 +4736,7 @@
         <v>11</v>
       </c>
       <c r="D175" s="3" t="s">
-        <v>148</v>
+        <v>113</v>
       </c>
       <c r="E175" s="3"/>
       <c r="F175" s="3"/>
@@ -4761,7 +4758,7 @@
         <v>12</v>
       </c>
       <c r="D176" s="3" t="s">
-        <v>149</v>
+        <v>114</v>
       </c>
       <c r="E176" s="3"/>
       <c r="F176" s="3"/>
@@ -4783,7 +4780,7 @@
         <v>6</v>
       </c>
       <c r="D177" s="3" t="s">
-        <v>150</v>
+        <v>115</v>
       </c>
       <c r="E177" s="3"/>
       <c r="F177" s="3"/>
@@ -4805,7 +4802,7 @@
         <v>7</v>
       </c>
       <c r="D178" s="3" t="s">
-        <v>151</v>
+        <v>116</v>
       </c>
       <c r="E178" s="3"/>
       <c r="F178" s="3"/>
@@ -4827,7 +4824,7 @@
         <v>8</v>
       </c>
       <c r="D179" s="3" t="s">
-        <v>152</v>
+        <v>117</v>
       </c>
       <c r="E179" s="3"/>
       <c r="F179" s="3"/>
@@ -4849,7 +4846,7 @@
         <v>9</v>
       </c>
       <c r="D180" s="3" t="s">
-        <v>153</v>
+        <v>118</v>
       </c>
       <c r="E180" s="3"/>
       <c r="F180" s="3"/>
@@ -5155,7 +5152,7 @@
       <c r="F195" s="3"/>
       <c r="G195" s="3"/>
       <c r="H195" s="6">
-        <f t="shared" ref="H195:H258" si="7">IF(A195&gt;DATE(2027,6,26),"",INT((A195-DATE(2026,8,31))/7)+1)</f>
+        <f t="shared" ref="H195:H258" si="7">IF(A195&gt;DATE(2027,6,25),"",INT((A195-DATE(2026,8,31))/7)+1)</f>
         <v>28</v>
       </c>
     </row>
@@ -5219,7 +5216,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="199" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+    <row r="199" spans="1:8" ht="32" x14ac:dyDescent="0.2">
       <c r="A199" s="2">
         <v>46463</v>
       </c>
@@ -5233,7 +5230,7 @@
       <c r="D199" s="3"/>
       <c r="E199" s="3"/>
       <c r="F199" s="3" t="s">
-        <v>50</v>
+        <v>128</v>
       </c>
       <c r="G199" s="3"/>
       <c r="H199" s="6">
@@ -5274,7 +5271,7 @@
       </c>
       <c r="D201" s="3"/>
       <c r="E201" s="3" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="F201" s="3"/>
       <c r="G201" s="3"/>
@@ -5395,7 +5392,7 @@
         <v>8</v>
       </c>
       <c r="D207" s="3" t="s">
-        <v>154</v>
+        <v>119</v>
       </c>
       <c r="E207" s="3"/>
       <c r="F207" s="3"/>
@@ -5417,7 +5414,7 @@
         <v>9</v>
       </c>
       <c r="D208" s="3" t="s">
-        <v>155</v>
+        <v>120</v>
       </c>
       <c r="E208" s="3"/>
       <c r="F208" s="3"/>
@@ -5439,7 +5436,7 @@
         <v>10</v>
       </c>
       <c r="D209" s="3" t="s">
-        <v>156</v>
+        <v>121</v>
       </c>
       <c r="E209" s="3"/>
       <c r="F209" s="3"/>
@@ -5449,7 +5446,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="210" spans="1:8" ht="96" x14ac:dyDescent="0.2">
+    <row r="210" spans="1:8" ht="128" x14ac:dyDescent="0.2">
       <c r="A210" s="2">
         <v>46474</v>
       </c>
@@ -5461,7 +5458,7 @@
         <v>11</v>
       </c>
       <c r="D210" s="3" t="s">
-        <v>157</v>
+        <v>132</v>
       </c>
       <c r="E210" s="3"/>
       <c r="F210" s="3"/>
@@ -5471,7 +5468,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="211" spans="1:8" ht="96" x14ac:dyDescent="0.2">
+    <row r="211" spans="1:8" ht="112" x14ac:dyDescent="0.2">
       <c r="A211" s="2">
         <v>46475</v>
       </c>
@@ -5483,7 +5480,7 @@
         <v>12</v>
       </c>
       <c r="D211" s="3" t="s">
-        <v>158</v>
+        <v>133</v>
       </c>
       <c r="E211" s="3"/>
       <c r="F211" s="3"/>
@@ -5505,7 +5502,7 @@
         <v>6</v>
       </c>
       <c r="D212" s="3" t="s">
-        <v>159</v>
+        <v>122</v>
       </c>
       <c r="E212" s="3"/>
       <c r="F212" s="3"/>
@@ -5710,7 +5707,7 @@
         <v>16</v>
       </c>
       <c r="E222" s="3" t="s">
-        <v>52</v>
+        <v>48</v>
       </c>
       <c r="F222" s="3"/>
       <c r="G222" s="3"/>
@@ -5913,7 +5910,7 @@
       <c r="D232" s="3"/>
       <c r="E232" s="3"/>
       <c r="F232" s="3" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
       <c r="G232" s="3"/>
       <c r="H232" s="6">
@@ -6056,7 +6053,7 @@
       </c>
       <c r="D239" s="3"/>
       <c r="E239" s="3" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
       <c r="F239" s="3"/>
       <c r="G239" s="3"/>
@@ -6077,7 +6074,7 @@
         <v>6</v>
       </c>
       <c r="D240" s="3" t="s">
-        <v>55</v>
+        <v>51</v>
       </c>
       <c r="E240" s="3"/>
       <c r="F240" s="3"/>
@@ -6087,7 +6084,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="241" spans="1:8" ht="64" x14ac:dyDescent="0.2">
+    <row r="241" spans="1:8" ht="80" x14ac:dyDescent="0.2">
       <c r="A241" s="2">
         <v>46505</v>
       </c>
@@ -6101,7 +6098,7 @@
       <c r="D241" s="3"/>
       <c r="E241" s="3"/>
       <c r="F241" s="3" t="s">
-        <v>56</v>
+        <v>129</v>
       </c>
       <c r="G241" s="3"/>
       <c r="H241" s="6">
@@ -6141,7 +6138,7 @@
         <v>9</v>
       </c>
       <c r="D243" s="3" t="s">
-        <v>57</v>
+        <v>52</v>
       </c>
       <c r="E243" s="3"/>
       <c r="F243" s="3"/>
@@ -6231,7 +6228,7 @@
       </c>
       <c r="E247" s="3"/>
       <c r="F247" s="3" t="s">
-        <v>58</v>
+        <v>53</v>
       </c>
       <c r="G247" s="3"/>
       <c r="H247" s="6">
@@ -6255,7 +6252,7 @@
       </c>
       <c r="E248" s="3"/>
       <c r="F248" s="3" t="s">
-        <v>59</v>
+        <v>54</v>
       </c>
       <c r="G248" s="3"/>
       <c r="H248" s="6">
@@ -6279,7 +6276,7 @@
       </c>
       <c r="E249" s="3"/>
       <c r="F249" s="3" t="s">
-        <v>60</v>
+        <v>55</v>
       </c>
       <c r="G249" s="3"/>
       <c r="H249" s="6">
@@ -6300,7 +6297,7 @@
       </c>
       <c r="D250" s="3"/>
       <c r="E250" s="3" t="s">
-        <v>61</v>
+        <v>56</v>
       </c>
       <c r="F250" s="3"/>
       <c r="G250" s="3"/>
@@ -6485,7 +6482,7 @@
       <c r="F259" s="3"/>
       <c r="G259" s="3"/>
       <c r="H259" s="6">
-        <f t="shared" ref="H259:H322" si="9">IF(A259&gt;DATE(2027,6,26),"",INT((A259-DATE(2026,8,31))/7)+1)</f>
+        <f t="shared" ref="H259:H322" si="9">IF(A259&gt;DATE(2027,6,25),"",INT((A259-DATE(2026,8,31))/7)+1)</f>
         <v>37</v>
       </c>
     </row>
@@ -6529,7 +6526,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="262" spans="1:8" ht="32" x14ac:dyDescent="0.2">
+    <row r="262" spans="1:8" ht="48" x14ac:dyDescent="0.2">
       <c r="A262" s="2">
         <v>46526</v>
       </c>
@@ -6543,7 +6540,7 @@
       <c r="D262" s="3"/>
       <c r="E262" s="3"/>
       <c r="F262" s="3" t="s">
-        <v>62</v>
+        <v>130</v>
       </c>
       <c r="G262" s="3"/>
       <c r="H262" s="6">
@@ -6645,7 +6642,7 @@
         <v>12</v>
       </c>
       <c r="D267" s="3" t="s">
-        <v>63</v>
+        <v>57</v>
       </c>
       <c r="E267" s="3"/>
       <c r="F267" s="3"/>
@@ -6668,7 +6665,7 @@
       </c>
       <c r="D268" s="3"/>
       <c r="E268" s="3" t="s">
-        <v>64</v>
+        <v>58</v>
       </c>
       <c r="F268" s="3"/>
       <c r="G268" s="3"/>
@@ -6813,7 +6810,7 @@
         <v>6</v>
       </c>
       <c r="D275" s="3" t="s">
-        <v>73</v>
+        <v>66</v>
       </c>
       <c r="E275" s="3"/>
       <c r="F275" s="3"/>
@@ -6957,7 +6954,7 @@
       <c r="D282" s="3"/>
       <c r="E282" s="3"/>
       <c r="F282" s="3" t="s">
-        <v>65</v>
+        <v>59</v>
       </c>
       <c r="G282" s="3"/>
       <c r="H282" s="6">
@@ -7097,7 +7094,7 @@
         <v>6</v>
       </c>
       <c r="D289" s="3" t="s">
-        <v>66</v>
+        <v>60</v>
       </c>
       <c r="E289" s="3"/>
       <c r="F289" s="3"/>
@@ -7140,7 +7137,7 @@
       </c>
       <c r="D291" s="3"/>
       <c r="E291" s="3" t="s">
-        <v>67</v>
+        <v>61</v>
       </c>
       <c r="F291" s="3"/>
       <c r="G291" s="3"/>
@@ -7161,7 +7158,7 @@
         <v>9</v>
       </c>
       <c r="D292" s="3" t="s">
-        <v>68</v>
+        <v>62</v>
       </c>
       <c r="E292" s="3"/>
       <c r="F292" s="3"/>
@@ -7223,11 +7220,11 @@
         <v>12</v>
       </c>
       <c r="D295" s="3" t="s">
-        <v>74</v>
+        <v>67</v>
       </c>
       <c r="E295" s="3"/>
       <c r="F295" s="3" t="s">
-        <v>69</v>
+        <v>63</v>
       </c>
       <c r="G295" s="3"/>
       <c r="H295" s="6">
@@ -7336,9 +7333,9 @@
       <c r="E300" s="3"/>
       <c r="F300" s="3"/>
       <c r="G300" s="3"/>
-      <c r="H300" s="6">
+      <c r="H300" s="6" t="str">
         <f t="shared" si="9"/>
-        <v>43</v>
+        <v/>
       </c>
     </row>
     <row r="301" spans="1:8" ht="16" x14ac:dyDescent="0.2">
@@ -7799,7 +7796,7 @@
       <c r="F323" s="3"/>
       <c r="G323" s="3"/>
       <c r="H323" s="6" t="str">
-        <f t="shared" ref="H323:H366" si="11">IF(A323&gt;DATE(2027,6,26),"",INT((A323-DATE(2026,8,31))/7)+1)</f>
+        <f t="shared" ref="H323:H366" si="11">IF(A323&gt;DATE(2027,6,25),"",INT((A323-DATE(2026,8,31))/7)+1)</f>
         <v/>
       </c>
     </row>
@@ -8323,7 +8320,7 @@
         <v/>
       </c>
     </row>
-    <row r="350" spans="1:8" ht="16" x14ac:dyDescent="0.2">
+    <row r="350" spans="1:8" ht="32" x14ac:dyDescent="0.2">
       <c r="A350" s="2">
         <v>46614</v>
       </c>
@@ -8334,7 +8331,9 @@
       <c r="C350" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="D350" s="3"/>
+      <c r="D350" s="3" t="s">
+        <v>134</v>
+      </c>
       <c r="E350" s="3"/>
       <c r="F350" s="3"/>
       <c r="G350" s="3"/>
@@ -8643,7 +8642,7 @@
         <v/>
       </c>
     </row>
-    <row r="366" spans="1:8" ht="80" x14ac:dyDescent="0.2">
+    <row r="366" spans="1:8" ht="112" x14ac:dyDescent="0.2">
       <c r="A366" s="2">
         <v>46630</v>
       </c>
@@ -8657,7 +8656,7 @@
       <c r="D366" s="3"/>
       <c r="E366" s="3"/>
       <c r="F366" s="3" t="s">
-        <v>70</v>
+        <v>131</v>
       </c>
       <c r="G366" s="3"/>
       <c r="H366" s="6" t="str">

</xml_diff>

<commit_message>
Add confectioner and baker student tournament
</commit_message>
<xml_diff>
--- a/kalendarz_dzienny_role_2026_2027.xlsx
+++ b/kalendarz_dzienny_role_2026_2027.xlsx
@@ -6174,7 +6174,11 @@
           <t>wtorek</t>
         </is>
       </c>
-      <c r="D233" s="3" t="n"/>
+      <c r="D233" s="3" t="inlineStr">
+        <is>
+          <t>Turniej na najlepszego ucznia w zawodzie cukiernik i piekarz</t>
+        </is>
+      </c>
       <c r="E233" s="3" t="n"/>
       <c r="F233" s="3" t="n"/>
       <c r="G233" s="3" t="n"/>
@@ -6196,7 +6200,11 @@
           <t>środa</t>
         </is>
       </c>
-      <c r="D234" s="3" t="n"/>
+      <c r="D234" s="3" t="inlineStr">
+        <is>
+          <t>Turniej na najlepszego ucznia w zawodzie cukiernik i piekarz</t>
+        </is>
+      </c>
       <c r="E234" s="3" t="n"/>
       <c r="F234" s="3" t="n"/>
       <c r="G234" s="3" t="n"/>
@@ -6220,7 +6228,8 @@
       </c>
       <c r="D235" s="3" t="inlineStr">
         <is>
-          <t>KLASY 5 TECHNIKUM: wystawienie ocen końcowych</t>
+          <t>KLASY 5 TECHNIKUM: wystawienie ocen końcowych
+Turniej na najlepszego ucznia w zawodzie cukiernik i piekarz</t>
         </is>
       </c>
       <c r="E235" s="3" t="n"/>

</xml_diff>

<commit_message>
Update September and school-year calendar entries
</commit_message>
<xml_diff>
--- a/kalendarz_dzienny_role_2026_2027.xlsx
+++ b/kalendarz_dzienny_role_2026_2027.xlsx
@@ -730,13 +730,13 @@
       <c r="D10" s="3" t="n"/>
       <c r="E10" s="3" t="inlineStr">
         <is>
-          <t>16:30 - KLASY 2-5 TECHNIKUM, KLASY 2-3 BS I st.: wychowawcy klas - zebrania z rodzicami
+          <t>17:00 - KLASY 2-5 TECHNIKUM, KLASY 2-3 BS I st.: wychowawcy klas - zebrania z rodzicami
 18:00 - zebranie Rady Rodziców</t>
         </is>
       </c>
       <c r="F10" s="3" t="inlineStr">
         <is>
-          <t>15:00/16:00 - RADA PEDAGOGICZNA: przedstawienie planu nadzoru pedagogicznego na rok szkolny 2026/2027</t>
+          <t>15:45 - RADA PEDAGOGICZNA: przedstawienie planu nadzoru pedagogicznego na rok szkolny 2026/2027</t>
         </is>
       </c>
       <c r="G10" s="3" t="n"/>
@@ -2897,10 +2897,15 @@
 Powód: praktyka zawodowa u pracodawcy – klasy 3 Technikum nie mają zajęć w szkole; pozostałe klasy uczą się normalnie.</t>
         </is>
       </c>
-      <c r="E101" s="3" t="n"/>
+      <c r="E101" s="3" t="inlineStr">
+        <is>
+          <t>17:00 - KLASY 5 TECHNIKUM: wychowawcy klas - zebrania z rodzicami na zakończenie I półrocza
+17:00 - 18:00 - POZOSTAŁE KLASY: wszyscy nauczyciele - konsultacje dla uczniów, w tym słuchaczy BS II st., i rodziców</t>
+        </is>
+      </c>
       <c r="F101" s="3" t="inlineStr">
         <is>
-          <t>15:00 - RADA PEDAGOGICZNA:
+          <t>15:45 - RADA PEDAGOGICZNA:
 1) klasyfikacyjna: KLASY 5 TECHNIKUM oraz 3 SEMESTR BS II st.
 2) szkoleniowa: szkolenie z procedur egzaminu zawodowego</t>
         </is>
@@ -2958,11 +2963,7 @@
 Powód: praktyka zawodowa u pracodawcy – klasy 3 Technikum nie mają zajęć w szkole; pozostałe klasy uczą się normalnie.</t>
         </is>
       </c>
-      <c r="E103" s="3" t="inlineStr">
-        <is>
-          <t>16:30 - KLASY 5 TECHNIKUM: wychowawcy klas - zebrania z rodzicami na zakończenie I półrocza / POZOSTAŁE KLASY: wszyscy nauczyciele - konsultacje dla uczniów, w tym słuchaczy BS II st., i rodziców - godz. 16:30 - 17:30</t>
-        </is>
-      </c>
+      <c r="E103" s="3" t="n"/>
       <c r="F103" s="3" t="n"/>
       <c r="G103" s="3" t="n"/>
       <c r="H103" s="6">
@@ -3846,7 +3847,11 @@
           <t>sobota</t>
         </is>
       </c>
-      <c r="D139" s="3" t="n"/>
+      <c r="D139" s="3" t="inlineStr">
+        <is>
+          <t>Studniówka</t>
+        </is>
+      </c>
       <c r="E139" s="3" t="n"/>
       <c r="F139" s="3" t="n"/>
       <c r="G139" s="3" t="n"/>
@@ -5922,12 +5927,13 @@
       </c>
       <c r="D222" s="3" t="inlineStr">
         <is>
-          <t>16:00 - KLASY 5 TECHNIKUM: wystawienie proponowanych ocen końcowych (maksymalnie do godz. 16:00)</t>
+          <t>KLASY 5 TECHNIKUM: wystawienie proponowanych ocen końcowych (maksymalnie do godz. 16:00)</t>
         </is>
       </c>
       <c r="E222" s="3" t="inlineStr">
         <is>
-          <t>16:30 - KLASY 5 TECHNIKUM: wychowawcy klas - zebrania z rodzicami / POZOSTAŁE KLASY: wszyscy nauczyciele - konsultacje dla uczniów, w tym słuchaczy BS II st., i rodziców - godz. 16:30 - 17:30</t>
+          <t>16:30 - KLASY 5 TECHNIKUM: wychowawcy klas - zebrania z rodzicami
+16:30 - 17:30 - POZOSTAŁE KLASY: wszyscy nauczyciele - konsultacje dla uczniów, w tym słuchaczy BS II st., i rodziców</t>
         </is>
       </c>
       <c r="F222" s="3" t="n"/>

</xml_diff>